<commit_message>
docs: update dedication file and add shared knowledge base document
</commit_message>
<xml_diff>
--- a/docs/Sprint 3/dedication/7-S3-dedication.xlsx
+++ b/docs/Sprint 3/dedication/7-S3-dedication.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\OneDrive\Escritorio\ispp s3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECC7031-EB51-4314-ADEC-9652B281DD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CDB1F25-91BF-47C9-8793-2A4991DB7315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{02C8C9D8-2F21-45BA-9A66-91BB45160C54}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="56">
   <si>
     <t>Nombre</t>
   </si>
@@ -209,120 +209,6 @@
   </si>
   <si>
     <t>Comentarios sobre DP</t>
-  </si>
-  <si>
-    <t>Nota: este score_final muestra los porcentajes ya ajustados en función de la carga temporal de las tareas cerradas</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>Ángel Mateos</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>Celia Suárez</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>Nicolás Gómez</t>
-  </si>
-  <si>
-    <t>Francisco De Castro</t>
-  </si>
-  <si>
-    <t>Alberto García</t>
-  </si>
-  <si>
-    <t>Ignacio Martínez</t>
-  </si>
-  <si>
-    <t>Carolina Murillo</t>
-  </si>
-  <si>
-    <t>Paula Suárez</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Javier Castilla</t>
-  </si>
-  <si>
-    <t>Carlos Gallero</t>
-  </si>
-  <si>
-    <t>Manuel J. Niza</t>
-  </si>
-  <si>
-    <t>Juan José Cardesa</t>
-  </si>
-  <si>
-    <t>Jesús García</t>
-  </si>
-  <si>
-    <t>Marta Recio</t>
-  </si>
-  <si>
-    <t>Olga Cantalejo</t>
-  </si>
-  <si>
-    <t>Javier Gutiérrez</t>
-  </si>
-  <si>
-    <t>Nuno del Pino</t>
-  </si>
-  <si>
-    <t>Alejandro de los Reyes</t>
-  </si>
-  <si>
-    <t>Pablo Pérez</t>
-  </si>
-  <si>
-    <t>Javier Soria</t>
-  </si>
-  <si>
-    <t>Miguel Regidor</t>
-  </si>
-  <si>
-    <t>score_final</t>
-  </si>
-  <si>
-    <t>Tareas cerradas</t>
-  </si>
-  <si>
-    <t>Tareas asignadas</t>
-  </si>
-  <si>
-    <t>H.Real</t>
-  </si>
-  <si>
-    <t>Equipo</t>
-  </si>
-  <si>
-    <t>Las horas posicionan a cada miembro alrededor de la media, mientras que el número de tareas y su complejidad temporal ajusta el resultado según la carga real asumida. Finalmente se garantiza que la media sea exactamente 100%.</t>
-  </si>
-  <si>
-    <t>score_final = score_base × (100 / media(score_base))</t>
-  </si>
-  <si>
-    <t>score_base = (H.Real / H_media × 100) + (t_cerradas − t_media) × 2</t>
-  </si>
-  <si>
-    <t>t_media = tareas cerradas totales / 21  = 5.95</t>
-  </si>
-  <si>
-    <t>H_media = H.Real total / 21  = 22.8h</t>
-  </si>
-  <si>
-    <t>Fórmula usada:</t>
-  </si>
-  <si>
-    <t>Estos resultados se ajustan manualmente, en acordancia con todo el grupo, en función de la carga temporal de las tareas asignadas a cada miembro (registradas en forma de tallas en el repositorio) , de manera que se alcanzan los porcentajes más justos para el score_final</t>
   </si>
 </sst>
 </file>
@@ -466,13 +352,13 @@
     <xf numFmtId="9" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -924,7 +810,7 @@
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
@@ -948,7 +834,7 @@
         <v>1</v>
       </c>
       <c r="F2" s="15">
-        <v>1.0354000000000001</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2"/>
     </row>
@@ -969,7 +855,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="15">
-        <v>0.98240000000000005</v>
+        <v>1</v>
       </c>
       <c r="G3" s="2"/>
     </row>
@@ -990,7 +876,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="15">
-        <v>0.95979999999999999</v>
+        <v>1</v>
       </c>
       <c r="G4" s="2"/>
     </row>
@@ -1011,7 +897,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="15">
-        <v>0.94140000000000001</v>
+        <v>1</v>
       </c>
       <c r="G5" s="2"/>
     </row>
@@ -1032,7 +918,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="15">
-        <v>1.0913999999999999</v>
+        <v>1</v>
       </c>
       <c r="G6" s="2"/>
     </row>
@@ -1053,7 +939,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="15">
-        <v>1.0533999999999999</v>
+        <v>1</v>
       </c>
       <c r="G7" s="2"/>
       <c r="I7" s="10"/>
@@ -1075,7 +961,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="15">
-        <v>0.96040000000000003</v>
+        <v>1</v>
       </c>
       <c r="G8" s="2"/>
     </row>
@@ -1096,7 +982,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="15">
-        <v>0.99739999999999995</v>
+        <v>1</v>
       </c>
       <c r="G9" s="2"/>
     </row>
@@ -1117,7 +1003,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="15">
-        <v>0.95440000000000003</v>
+        <v>1</v>
       </c>
       <c r="G10" s="2"/>
     </row>
@@ -1138,7 +1024,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="15">
-        <v>0.93240000000000001</v>
+        <v>1</v>
       </c>
       <c r="G11" s="2"/>
     </row>
@@ -1159,7 +1045,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="15">
-        <v>1.0364</v>
+        <v>1</v>
       </c>
       <c r="G12" s="2"/>
     </row>
@@ -1180,7 +1066,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="15">
-        <v>0.95440000000000003</v>
+        <v>1</v>
       </c>
       <c r="G13" s="2"/>
     </row>
@@ -1201,7 +1087,7 @@
         <v>1</v>
       </c>
       <c r="F14" s="15">
-        <v>0.88539999999999996</v>
+        <v>1</v>
       </c>
       <c r="G14" s="2"/>
     </row>
@@ -1222,7 +1108,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="15">
-        <v>0.95840000000000003</v>
+        <v>1</v>
       </c>
       <c r="G15" s="2"/>
     </row>
@@ -1243,7 +1129,7 @@
         <v>1</v>
       </c>
       <c r="F16" s="15">
-        <v>0.97340000000000004</v>
+        <v>1</v>
       </c>
       <c r="G16" s="2"/>
     </row>
@@ -1264,7 +1150,7 @@
         <v>1</v>
       </c>
       <c r="F17" s="15">
-        <v>1.0973999999999999</v>
+        <v>1</v>
       </c>
       <c r="G17" s="12"/>
     </row>
@@ -1285,7 +1171,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="15">
-        <v>1.0344</v>
+        <v>1</v>
       </c>
       <c r="G18" s="2"/>
     </row>
@@ -1306,7 +1192,7 @@
         <v>1</v>
       </c>
       <c r="F19" s="15">
-        <v>1.1404000000000001</v>
+        <v>1</v>
       </c>
       <c r="G19" s="2"/>
     </row>
@@ -1327,7 +1213,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="15">
-        <v>1.1334</v>
+        <v>1</v>
       </c>
       <c r="G20" s="2"/>
     </row>
@@ -1348,9 +1234,9 @@
         <v>1</v>
       </c>
       <c r="F21" s="15">
-        <v>0.91959999999999997</v>
-      </c>
-      <c r="G21" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="G21"/>
     </row>
     <row r="22" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
@@ -1369,7 +1255,7 @@
         <v>1</v>
       </c>
       <c r="F22" s="15">
-        <v>0.95840000000000003</v>
+        <v>1</v>
       </c>
       <c r="G22" s="2"/>
     </row>
@@ -1441,34 +1327,34 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
     </row>
     <row r="34" spans="4:4" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" spans="4:4" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1549,493 +1435,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{513504E1-60A0-43FB-A9A1-0E8466BB8143}">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" customWidth="1"/>
   </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B13" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" t="s">
-        <v>84</v>
-      </c>
-      <c r="E13" t="s">
-        <v>83</v>
-      </c>
-      <c r="F13" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>81</v>
-      </c>
-      <c r="B14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C14">
-        <v>31.9</v>
-      </c>
-      <c r="D14">
-        <v>5</v>
-      </c>
-      <c r="E14">
-        <v>5</v>
-      </c>
-      <c r="F14" s="15">
-        <v>1.1404000000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>80</v>
-      </c>
-      <c r="B15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15">
-        <v>29.1</v>
-      </c>
-      <c r="D15">
-        <v>8</v>
-      </c>
-      <c r="E15">
-        <v>8</v>
-      </c>
-      <c r="F15" s="15">
-        <v>1.1334</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>79</v>
-      </c>
-      <c r="B16" t="s">
-        <v>57</v>
-      </c>
-      <c r="C16">
-        <v>26.6</v>
-      </c>
-      <c r="D16">
-        <v>8</v>
-      </c>
-      <c r="E16">
-        <v>8</v>
-      </c>
-      <c r="F16" s="15">
-        <v>1.0973999999999999</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>78</v>
-      </c>
-      <c r="B17" t="s">
-        <v>68</v>
-      </c>
-      <c r="C17">
-        <v>26.3</v>
-      </c>
-      <c r="D17">
-        <v>8</v>
-      </c>
-      <c r="E17">
-        <v>8</v>
-      </c>
-      <c r="F17" s="15">
-        <v>1.0913999999999999</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>77</v>
-      </c>
-      <c r="B18" t="s">
-        <v>68</v>
-      </c>
-      <c r="C18">
-        <v>24.6</v>
-      </c>
-      <c r="D18">
-        <v>7</v>
-      </c>
-      <c r="E18">
-        <v>7</v>
-      </c>
-      <c r="F18" s="15">
-        <v>1.0533999999999999</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>76</v>
-      </c>
-      <c r="B19" t="s">
-        <v>68</v>
-      </c>
-      <c r="C19">
-        <v>24.5</v>
-      </c>
-      <c r="D19">
-        <v>6</v>
-      </c>
-      <c r="E19">
-        <v>6</v>
-      </c>
-      <c r="F19" s="15">
-        <v>1.0364</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>75</v>
-      </c>
-      <c r="B20" t="s">
-        <v>59</v>
-      </c>
-      <c r="C20">
-        <v>22.7</v>
-      </c>
-      <c r="D20">
-        <v>10</v>
-      </c>
-      <c r="E20">
-        <v>10</v>
-      </c>
-      <c r="F20" s="15">
-        <v>1.0354000000000001</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>74</v>
-      </c>
-      <c r="B21" t="s">
-        <v>59</v>
-      </c>
-      <c r="C21">
-        <v>21.9</v>
-      </c>
-      <c r="D21">
-        <v>11</v>
-      </c>
-      <c r="E21">
-        <v>11</v>
-      </c>
-      <c r="F21" s="15">
-        <v>1.0344</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>73</v>
-      </c>
-      <c r="B22" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22">
-        <v>24</v>
-      </c>
-      <c r="D22">
-        <v>4</v>
-      </c>
-      <c r="E22">
-        <v>4</v>
-      </c>
-      <c r="F22" s="15">
-        <v>0.99739999999999995</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>72</v>
-      </c>
-      <c r="B23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C23">
-        <v>21.4</v>
-      </c>
-      <c r="D23">
-        <v>7</v>
-      </c>
-      <c r="E23">
-        <v>7</v>
-      </c>
-      <c r="F23" s="15">
-        <v>0.98240000000000005</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>71</v>
-      </c>
-      <c r="B24" t="s">
-        <v>61</v>
-      </c>
-      <c r="C24">
-        <v>20.5</v>
-      </c>
-      <c r="D24">
-        <v>8</v>
-      </c>
-      <c r="E24">
-        <v>8</v>
-      </c>
-      <c r="F24" s="15">
-        <v>0.97340000000000004</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>70</v>
-      </c>
-      <c r="B25" t="s">
-        <v>57</v>
-      </c>
-      <c r="C25">
-        <v>21</v>
-      </c>
-      <c r="D25">
-        <v>5</v>
-      </c>
-      <c r="E25">
-        <v>5</v>
-      </c>
-      <c r="F25" s="15">
-        <v>0.96040000000000003</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>69</v>
-      </c>
-      <c r="B26" t="s">
-        <v>68</v>
-      </c>
-      <c r="C26">
-        <v>20.9</v>
-      </c>
-      <c r="D26">
-        <v>5</v>
-      </c>
-      <c r="E26">
-        <v>5</v>
-      </c>
-      <c r="F26" s="15">
-        <v>0.95979999999999999</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>67</v>
-      </c>
-      <c r="B27" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27">
-        <v>20.5</v>
-      </c>
-      <c r="D27">
-        <v>6</v>
-      </c>
-      <c r="E27">
-        <v>6</v>
-      </c>
-      <c r="F27" s="15">
-        <v>0.95840000000000003</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>66</v>
-      </c>
-      <c r="B28" t="s">
-        <v>59</v>
-      </c>
-      <c r="C28">
-        <v>20.8</v>
-      </c>
-      <c r="D28">
-        <v>5</v>
-      </c>
-      <c r="E28">
-        <v>5</v>
-      </c>
-      <c r="F28" s="15">
-        <v>0.95840000000000003</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>65</v>
-      </c>
-      <c r="B29" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29">
-        <v>21.2</v>
-      </c>
-      <c r="D29">
-        <v>4</v>
-      </c>
-      <c r="E29">
-        <v>4</v>
-      </c>
-      <c r="F29" s="15">
-        <v>0.95440000000000003</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>64</v>
-      </c>
-      <c r="B30" t="s">
-        <v>57</v>
-      </c>
-      <c r="C30">
-        <v>20.7</v>
-      </c>
-      <c r="D30">
-        <v>5</v>
-      </c>
-      <c r="E30">
-        <v>5</v>
-      </c>
-      <c r="F30" s="15">
-        <v>0.95440000000000003</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>63</v>
-      </c>
-      <c r="B31" t="s">
-        <v>57</v>
-      </c>
-      <c r="C31">
-        <v>20.2</v>
-      </c>
-      <c r="D31">
-        <v>5</v>
-      </c>
-      <c r="E31">
-        <v>5</v>
-      </c>
-      <c r="F31" s="15">
-        <v>0.94140000000000001</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32" t="s">
-        <v>61</v>
-      </c>
-      <c r="C32">
-        <v>21.7</v>
-      </c>
-      <c r="D32">
-        <v>4</v>
-      </c>
-      <c r="E32">
-        <v>3</v>
-      </c>
-      <c r="F32" s="15">
-        <v>0.93240000000000001</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>60</v>
-      </c>
-      <c r="B33" t="s">
-        <v>59</v>
-      </c>
-      <c r="C33">
-        <v>20.2</v>
-      </c>
-      <c r="D33">
-        <v>4</v>
-      </c>
-      <c r="E33">
-        <v>3</v>
-      </c>
-      <c r="F33" s="15">
-        <v>0.91959999999999997</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>58</v>
-      </c>
-      <c r="B34" t="s">
-        <v>57</v>
-      </c>
-      <c r="C34">
-        <v>18.2</v>
-      </c>
-      <c r="D34">
-        <v>2</v>
-      </c>
-      <c r="E34">
-        <v>2</v>
-      </c>
-      <c r="F34" s="15">
-        <v>0.88539999999999996</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="F36" t="s">
-        <v>56</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2050,23 +1455,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="1a6abb52-502d-48a4-9af4-2c760790d608" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101004DDB13F6C19E524F885E2684B5F16C1D" ma:contentTypeVersion="10" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="85bcce37b1c78db65bbe0822d8028ee1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="1a6abb52-502d-48a4-9af4-2c760790d608" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="548aeb65dc532bcd5edd0448b207d0ab" ns3:_="">
     <xsd:import namespace="1a6abb52-502d-48a4-9af4-2c760790d608"/>
@@ -2248,10 +1636,37 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="1a6abb52-502d-48a4-9af4-2c760790d608" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F4B272D-551A-4AF9-B220-C688C9745ED1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86F6973B-E301-4E76-B65C-A7477A18457B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1a6abb52-502d-48a4-9af4-2c760790d608"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2267,19 +1682,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86F6973B-E301-4E76-B65C-A7477A18457B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F4B272D-551A-4AF9-B220-C688C9745ED1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1a6abb52-502d-48a4-9af4-2c760790d608"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>